<commit_message>
test(defect-log): record 7 rigorous bugs discovered via multi-tool deep boundary probing
</commit_message>
<xml_diff>
--- a/Testing/04_TaiLieu_Va_BaoCao_KiemThu/BANG_KE_HOACH_VA_KICH_BAN_KIEM_THU_137_TC.xlsx
+++ b/Testing/04_TaiLieu_Va_BaoCao_KiemThu/BANG_KE_HOACH_VA_KICH_BAN_KIEM_THU_137_TC.xlsx
@@ -1473,7 +1473,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:E33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.6640625" customWidth="1" min="1" max="1"/>
     <col width="32.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -1855,7 +1855,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="I6" s="24" t="inlineStr">
         <is>
-          <t>Tài khoản thường (User) cố tình truy cập /Admin bị chặn và trả về 403 Forbidden / Access Denied.</t>
-        </is>
-      </c>
-      <c r="J6" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 302 Found, chuyển hướng (Redirect) về /Auth/Login?ReturnUrl=%2FAdmin</t>
+        </is>
+      </c>
+      <c r="J6" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K6" s="26" t="inlineStr">
@@ -2059,7 +2059,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="L6" s="35" t="n"/>
+      <c r="L6" s="35" t="inlineStr">
+        <is>
+          <t>BUG_003</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="55.2" customHeight="1">
       <c r="A7" s="20" t="n">
@@ -2449,12 +2453,12 @@
       </c>
       <c r="I13" s="24" t="inlineStr">
         <is>
-          <t>Chỉnh sửa thông tin và xóa bài cờ thế trong CMS cập nhật chính xác.</t>
-        </is>
-      </c>
-      <c r="J13" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 200 OK (hoặc redirect thành công) gây sai lệch trạng thái CMS</t>
+        </is>
+      </c>
+      <c r="J13" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K13" s="27" t="inlineStr">
@@ -2462,7 +2466,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="L13" s="35" t="n"/>
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>BUG_007</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="55.2" customHeight="1">
       <c r="A14" s="20" t="n">
@@ -2662,7 +2670,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -3463,7 +3471,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6.6640625" customWidth="1" min="1" max="1"/>
     <col width="12.6640625" customWidth="1" min="2" max="2"/>
@@ -3565,12 +3573,12 @@
       </c>
       <c r="C5" s="35" t="inlineStr">
         <is>
-          <t>Cho phép đăng ký mật khẩu yếu dưới 6 ký tự</t>
+          <t>Cho phép đăng ký mật khẩu yếu dưới 6 ký tự qua API</t>
         </is>
       </c>
       <c r="D5" s="35" t="inlineStr">
         <is>
-          <t>Xác thực &amp; Tài khoản</t>
+          <t>Xác thực &amp; Tài khoản (04_TC_Auth_Profile)</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
@@ -3585,17 +3593,19 @@
       </c>
       <c r="G5" s="35" t="inlineStr">
         <is>
-          <t>Gửi password 123</t>
+          <t>1. Gửi POST /api/auth/register
+2. Body chứa password = '123'
+3. Kiểm tra mã phản hồi</t>
         </is>
       </c>
       <c r="H5" s="35" t="inlineStr">
         <is>
-          <t>Chặn lỗi mật khẩu ngắn</t>
+          <t>HTTP 400 Bad Request, báo lỗi mật khẩu phải &gt;= 6 ký tự</t>
         </is>
       </c>
       <c r="I5" s="35" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>HTTP 200 OK, hệ thống tạo tài khoản thành công với mật khẩu 3 ký tự</t>
         </is>
       </c>
       <c r="J5" s="35" t="inlineStr">
@@ -3608,7 +3618,7 @@
           <t>Tester độc lập</t>
         </is>
       </c>
-      <c r="L5" s="64" t="inlineStr">
+      <c r="L5" s="63" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3623,16 +3633,58 @@
           <t>BUG_002</t>
         </is>
       </c>
-      <c r="C6" s="35" t="n"/>
-      <c r="D6" s="35" t="n"/>
-      <c r="E6" s="35" t="n"/>
-      <c r="F6" s="35" t="n"/>
-      <c r="G6" s="35" t="n"/>
-      <c r="H6" s="35" t="n"/>
-      <c r="I6" s="35" t="n"/>
-      <c r="J6" s="35" t="n"/>
-      <c r="K6" s="35" t="n"/>
-      <c r="L6" s="20" t="n"/>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Thiếu Regex kiểm tra định dạng Email khi đăng ký tài khoản</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Xác thực &amp; Tài khoản (04_TC_Auth_Profile)</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr">
+        <is>
+          <t>P2 - Major</t>
+        </is>
+      </c>
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /api/auth/register
+2. Body email = 'not_an_email_at_all' (không có @ và domain)
+3. Bấm đăng ký</t>
+        </is>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request, từ chối định dạng email không hợp lệ</t>
+        </is>
+      </c>
+      <c r="I6" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, tài khoản vẫn được tạo với email rác trong CSDL</t>
+        </is>
+      </c>
+      <c r="J6" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_AUTH_001.png</t>
+        </is>
+      </c>
+      <c r="K6" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L6" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="28.05" customHeight="1">
       <c r="A7" s="20" t="n">
@@ -3643,16 +3695,57 @@
           <t>BUG_003</t>
         </is>
       </c>
-      <c r="C7" s="35" t="n"/>
-      <c r="D7" s="35" t="n"/>
-      <c r="E7" s="35" t="n"/>
-      <c r="F7" s="35" t="n"/>
-      <c r="G7" s="35" t="n"/>
-      <c r="H7" s="35" t="n"/>
-      <c r="I7" s="35" t="n"/>
-      <c r="J7" s="35" t="n"/>
-      <c r="K7" s="35" t="n"/>
-      <c r="L7" s="20" t="n"/>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>Truy cập /Admin khi chưa phân quyền trả về 302 Redirect thay vì 403 Forbidden</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>Phân hệ Quản trị viên (10_TC_Admin_System)</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>P2 - Major</t>
+        </is>
+      </c>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G7" s="35" t="inlineStr">
+        <is>
+          <t>1. Người dùng chưa đăng nhập hoặc role User truy cập URL /Admin
+2. Kiểm tra HTTP Status Code trả về</t>
+        </is>
+      </c>
+      <c r="H7" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 403 Forbidden (hoặc trang Access Denied 403)</t>
+        </is>
+      </c>
+      <c r="I7" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 302 Found, chuyển hướng (Redirect) về /Auth/Login?ReturnUrl=%2FAdmin</t>
+        </is>
+      </c>
+      <c r="J7" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_ADM_002.png</t>
+        </is>
+      </c>
+      <c r="K7" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L7" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28.05" customHeight="1">
       <c r="A8" s="20" t="n">
@@ -3663,16 +3756,58 @@
           <t>BUG_004</t>
         </is>
       </c>
-      <c r="C8" s="35" t="n"/>
-      <c r="D8" s="35" t="n"/>
-      <c r="E8" s="35" t="n"/>
-      <c r="F8" s="35" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="35" t="n"/>
-      <c r="I8" s="35" t="n"/>
-      <c r="J8" s="35" t="n"/>
-      <c r="K8" s="35" t="n"/>
-      <c r="L8" s="20" t="n"/>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>Vẫn cho phép đi quân cờ sau khi người chơi đã bấm Xin hàng (Surrender)</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>Đấu trực tuyến &amp; Vận hành ván cờ (07_TC_Online_SignalR)</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>P1 - Blocker</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G8" s="35" t="inlineStr">
+        <is>
+          <t>1. Tạo ván cờ mới
+2. Bên Đỏ gọi POST /api/games/{id}/surrender
+3. Bên Đỏ tiếp tục gửi nước đi POST /api/games/{id}/moves</t>
+        </is>
+      </c>
+      <c r="H8" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request, ván cờ đã kết thúc không thể đi thêm nước cờ</t>
+        </is>
+      </c>
+      <c r="I8" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, server tiếp tục nhận nước cờ và đổi trạng thái về InProgress</t>
+        </is>
+      </c>
+      <c r="J8" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_ONL_015.png</t>
+        </is>
+      </c>
+      <c r="K8" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L8" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28.05" customHeight="1">
       <c r="A9" s="20" t="n">
@@ -3683,16 +3818,58 @@
           <t>BUG_005</t>
         </is>
       </c>
-      <c r="C9" s="35" t="n"/>
-      <c r="D9" s="35" t="n"/>
-      <c r="E9" s="35" t="n"/>
-      <c r="F9" s="35" t="n"/>
-      <c r="G9" s="35" t="n"/>
-      <c r="H9" s="35" t="n"/>
-      <c r="I9" s="35" t="n"/>
-      <c r="J9" s="35" t="n"/>
-      <c r="K9" s="35" t="n"/>
-      <c r="L9" s="20" t="n"/>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Cấp Chứng chỉ tốt nghiệp cho người dùng chưa hoàn thành khóa học (0% tiến độ)</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>Học viện &amp; Kỳ phổ (09_TC_Course_Master)</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>P2 - Major</t>
+        </is>
+      </c>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G9" s="35" t="inlineStr">
+        <is>
+          <t>1. Người dùng mới tạo chưa học bài nào
+2. Truy cập trực tiếp /Course/Certificate?courseId=1
+3. Kiểm tra trang hiển thị</t>
+        </is>
+      </c>
+      <c r="H9" s="35" t="inlineStr">
+        <is>
+          <t>Từ chối cấp chứng chỉ, thông báo học viên cần hoàn thành 100% khóa học</t>
+        </is>
+      </c>
+      <c r="I9" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, hệ thống vẫn kết xuất chứng chỉ tốt nghiệp hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="J9" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_COU_009.png</t>
+        </is>
+      </c>
+      <c r="K9" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L9" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28.05" customHeight="1">
       <c r="A10" s="20" t="n">
@@ -3703,16 +3880,57 @@
           <t>BUG_006</t>
         </is>
       </c>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="35" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="35" t="n"/>
-      <c r="I10" s="35" t="n"/>
-      <c r="J10" s="35" t="n"/>
-      <c r="K10" s="35" t="n"/>
-      <c r="L10" s="20" t="n"/>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>API tiến độ khóa học không chặn ngưỡng điểm Quiz (Chấp nhận điểm 999999%)</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>Học viện &amp; Kỳ phổ (09_TC_Course_Master)</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
+        <is>
+          <t>P3 - Minor</t>
+        </is>
+      </c>
+      <c r="F10" s="35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G10" s="35" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /api/courses/progress với quizScore = 999999
+2. Kiểm tra phản hồi máy chủ</t>
+        </is>
+      </c>
+      <c r="H10" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request, điểm số Quiz phải nằm trong khoảng 0 đến 100%</t>
+        </is>
+      </c>
+      <c r="I10" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK, máy chủ lưu nguyên vẹn bestQuizScore = 999999</t>
+        </is>
+      </c>
+      <c r="J10" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_COU_008.png</t>
+        </is>
+      </c>
+      <c r="K10" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L10" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28.05" customHeight="1">
       <c r="A11" s="20" t="n">
@@ -3723,16 +3941,57 @@
           <t>BUG_007</t>
         </is>
       </c>
-      <c r="C11" s="35" t="n"/>
-      <c r="D11" s="35" t="n"/>
-      <c r="E11" s="35" t="n"/>
-      <c r="F11" s="35" t="n"/>
-      <c r="G11" s="35" t="n"/>
-      <c r="H11" s="35" t="n"/>
-      <c r="I11" s="35" t="n"/>
-      <c r="J11" s="35" t="n"/>
-      <c r="K11" s="35" t="n"/>
-      <c r="L11" s="20" t="n"/>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>Chức năng Xóa bài cờ thế trong Admin trả về HTTP 200 khi ID không tồn tại</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>Phân hệ Quản trị viên (10_TC_Admin_System)</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="inlineStr">
+        <is>
+          <t>P3 - Minor</t>
+        </is>
+      </c>
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G11" s="35" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /Admin/DeletePuzzle với id = 999999 không có trong CSDL
+2. Kiểm tra mã phản hồi</t>
+        </is>
+      </c>
+      <c r="H11" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 404 Not Found hoặc báo lỗi không tìm thấy bài cờ cần xóa</t>
+        </is>
+      </c>
+      <c r="I11" s="35" t="inlineStr">
+        <is>
+          <t>HTTP 200 OK (hoặc redirect thành công) gây sai lệch trạng thái CMS</t>
+        </is>
+      </c>
+      <c r="J11" s="35" t="inlineStr">
+        <is>
+          <t>E2E_SCREENSHOTS/TC_ADM_009.png</t>
+        </is>
+      </c>
+      <c r="K11" s="35" t="inlineStr">
+        <is>
+          <t>Tester độc lập</t>
+        </is>
+      </c>
+      <c r="L11" s="63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28.05" customHeight="1">
       <c r="A12" s="20" t="n">
@@ -4122,7 +4381,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:E24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.6640625" customWidth="1" min="1" max="1"/>
     <col width="24.6640625" customWidth="1" min="2" max="2"/>
@@ -4444,7 +4703,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:J19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.6640625" customWidth="1" min="1" max="1"/>
     <col width="6.6640625" customWidth="1" min="2" max="2"/>
@@ -4945,7 +5204,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -5082,12 +5341,12 @@
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>Đăng ký thành công tài khoản kythu_1793112405, cấp PlayerId và Token phiên.</t>
-        </is>
-      </c>
-      <c r="J5" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 200 OK, tài khoản vẫn được tạo với email rác trong CSDL</t>
+        </is>
+      </c>
+      <c r="J5" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K5" s="16" t="inlineStr">
@@ -5095,7 +5354,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="L5" s="13" t="n"/>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>BUG_002</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="52.8" customHeight="1">
       <c r="A6" s="11" t="n">
@@ -5256,7 +5519,7 @@
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>Không chặn pass ngắn: HTTP 200</t>
+          <t>HTTP 200 OK, hệ thống tạo tài khoản thành công với mật khẩu 3 ký tự</t>
         </is>
       </c>
       <c r="J8" s="63" t="inlineStr">
@@ -6046,7 +6309,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -7644,7 +7907,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -8789,7 +9052,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -9723,12 +9986,12 @@
       </c>
       <c r="I19" s="24" t="inlineStr">
         <is>
-          <t>Người chơi bấm Xin hàng (Resign): Hệ thống xử thua ngay lập tức và cập nhật Elo.</t>
-        </is>
-      </c>
-      <c r="J19" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 200 OK, server tiếp tục nhận nước cờ và đổi trạng thái về InProgress</t>
+        </is>
+      </c>
+      <c r="J19" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K19" s="26" t="inlineStr">
@@ -9736,7 +9999,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="L19" s="35" t="n"/>
+      <c r="L19" s="35" t="inlineStr">
+        <is>
+          <t>BUG_004</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="41.4" customFormat="1" customHeight="1" s="28">
       <c r="A20" s="20" t="n">
@@ -10045,7 +10312,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -11074,7 +11341,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.6640625" customWidth="1" min="1" max="1"/>
     <col width="15.6640625" customWidth="1" min="2" max="2"/>
@@ -11607,12 +11874,12 @@
       </c>
       <c r="I12" s="24" t="inlineStr">
         <is>
-          <t>Lưu tiến độ qua API /api/courses/progress: Ghi nhận isCompleted = true và cập nhật % khóa học.</t>
-        </is>
-      </c>
-      <c r="J12" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 200 OK, máy chủ lưu nguyên vẹn bestQuizScore = 999999</t>
+        </is>
+      </c>
+      <c r="J12" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K12" s="26" t="inlineStr">
@@ -11620,7 +11887,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="L12" s="35" t="n"/>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>BUG_006</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="55.2" customFormat="1" customHeight="1" s="28">
       <c r="A13" s="20" t="n">
@@ -11664,12 +11935,12 @@
       </c>
       <c r="I13" s="24" t="inlineStr">
         <is>
-          <t>Hoàn thành 100% khóa học: Cấp Chứng chỉ tốt nghiệp điện tử trang trọng kèm mã xác thực.</t>
-        </is>
-      </c>
-      <c r="J13" s="62" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>HTTP 200 OK, hệ thống vẫn kết xuất chứng chỉ tốt nghiệp hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="J13" s="63" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="K13" s="27" t="inlineStr">
@@ -11677,7 +11948,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="L13" s="35" t="n"/>
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>BUG_005</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="55.2" customFormat="1" customHeight="1" s="28">
       <c r="A14" s="20" t="n">

</xml_diff>